<commit_message>
chore: update finance tracking, API types, and company settings
- Update Techmigos finance tracking spreadsheet
- Add InsForge migrations for finance proof attachments, invoice tracking, company settings, and sign URLs
- Update package dependencies
- Refresh client and company pages

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Techmigos Fin Track.xlsx
+++ b/Techmigos Fin Track.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="7"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -457,40 +457,44 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -498,15 +502,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -514,39 +518,39 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -554,15 +558,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -801,34 +805,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="1f497d"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="eeece1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="4f81bd"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="c0504d"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="9bbb59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="8064a2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="4bacc6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="f79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="0000ff"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -974,107 +978,107 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G13"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="30.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="2" width="30.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
-        <v>46073</v>
-      </c>
-      <c r="B2" s="0" t="s">
+        <v>46086</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="5" t="n">
-        <v>7000</v>
-      </c>
-    </row>
-    <row r="3" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G2" s="6" t="n">
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="3" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
-        <v>46080</v>
-      </c>
-      <c r="B3" s="0" t="s">
+        <v>46112</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="5" t="n">
-        <v>9000</v>
+      <c r="G3" s="6" t="n">
+        <v>8700</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="A4" s="8" t="n">
         <v>46086</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="9" t="n">
         <v>452</v>
       </c>
     </row>
@@ -1082,137 +1086,137 @@
       <c r="A5" s="1" t="n">
         <v>46103</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="5" t="n">
+      <c r="G5" s="6" t="n">
         <v>2500</v>
       </c>
     </row>
-    <row r="6" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>46104</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="5" t="n">
-        <v>2800</v>
+      <c r="G6" s="6" t="n">
+        <v>2696</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="8" t="n">
         <v>46136</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="9" t="n">
+      <c r="G7" s="10" t="n">
         <v>711</v>
       </c>
     </row>
-    <row r="8" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>46137</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="6" t="n">
         <v>1700</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="8" t="n">
         <v>46162</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>413</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="11" t="n">
         <v>46032</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="11" t="s">
+      <c r="F10" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="13" t="n">
         <v>350</v>
       </c>
     </row>
@@ -1220,68 +1224,68 @@
       <c r="A11" s="1" t="n">
         <v>46143</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="6" t="n">
         <v>250</v>
       </c>
     </row>
-    <row r="12" s="6" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" s="7" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>21000</v>
+      <c r="G12" s="14" t="n">
+        <v>20407.52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
+      <c r="A13" s="8" t="n">
         <v>46178</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="9" t="n">
         <v>478</v>
       </c>
     </row>
@@ -1305,41 +1309,41 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="B1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="E1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="16" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1347,25 +1351,25 @@
       <c r="A2" s="1" t="n">
         <v>46055</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="5" t="n">
+      <c r="H2" s="6" t="n">
         <v>20000</v>
       </c>
     </row>
@@ -1373,25 +1377,25 @@
       <c r="A3" s="1" t="n">
         <v>46058</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="H3" s="6" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -1399,25 +1403,25 @@
       <c r="A4" s="1" t="n">
         <v>46175</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="H4" s="6" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -1425,25 +1429,25 @@
       <c r="A5" s="1" t="n">
         <v>46175</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="H5" s="6" t="n">
         <v>11499</v>
       </c>
     </row>
@@ -1451,25 +1455,25 @@
       <c r="A6" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="5" t="n">
+      <c r="H6" s="6" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -1493,41 +1497,41 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="16" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="27.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="17" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="C1" s="18" t="s">
+      <c r="C1" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="D1" s="18" t="s">
+      <c r="D1" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="18" t="s">
+      <c r="F1" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="18" t="s">
+      <c r="G1" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="19" t="s">
+      <c r="H1" s="20" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1535,25 +1539,25 @@
       <c r="A2" s="1" t="n">
         <v>46174</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="H2" s="16" t="n">
+      <c r="H2" s="17" t="n">
         <v>1499</v>
       </c>
     </row>
@@ -1577,41 +1581,41 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="16" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="17" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="22" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="23" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1619,25 +1623,25 @@
       <c r="A2" s="1" t="n">
         <v>46149</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H2" s="16" t="n">
+      <c r="H2" s="17" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -1645,25 +1649,25 @@
       <c r="A3" s="1" t="n">
         <v>46149</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H3" s="23" t="n">
+      <c r="H3" s="24" t="n">
         <v>3000</v>
       </c>
     </row>
@@ -1671,25 +1675,25 @@
       <c r="A4" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G4" s="0" t="s">
+      <c r="G4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="16" t="n">
+      <c r="H4" s="17" t="n">
         <v>4000</v>
       </c>
     </row>
@@ -1697,25 +1701,25 @@
       <c r="A5" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G5" s="0" t="s">
+      <c r="G5" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <v>2500</v>
       </c>
     </row>
@@ -1723,25 +1727,25 @@
       <c r="A6" s="1" t="n">
         <v>46186</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="G6" s="0" t="s">
+      <c r="G6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>1000</v>
       </c>
     </row>
@@ -1765,67 +1769,67 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.25" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="35.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="16" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="40.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="35.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="17" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="2" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="2" width="40.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16381" style="2" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="25" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="24" t="s">
+      <c r="C1" s="25" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="24" t="s">
+      <c r="D1" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="25" t="s">
+      <c r="E1" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="G1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="H1" s="25" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="26" t="s">
+      <c r="I1" s="27" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="25" t="s">
         <v>84</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="K1" s="25" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E2" s="1" t="n">
@@ -1834,33 +1838,33 @@
       <c r="F2" s="1" t="n">
         <v>46193</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="I2" s="16" t="n">
+      <c r="I2" s="17" t="n">
         <v>30000</v>
       </c>
-      <c r="J2" s="0" t="n">
+      <c r="J2" s="2" t="n">
         <v>90</v>
       </c>
-      <c r="K2" s="0" t="s">
+      <c r="K2" s="2" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="2" t="s">
         <v>28</v>
       </c>
       <c r="E3" s="1" t="n">
@@ -1869,19 +1873,19 @@
       <c r="F3" s="1" t="n">
         <v>46194</v>
       </c>
-      <c r="G3" s="0" t="s">
+      <c r="G3" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="I3" s="16" t="n">
+      <c r="I3" s="17" t="n">
         <v>40000</v>
       </c>
-      <c r="J3" s="0" t="n">
+      <c r="J3" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="K3" s="0" t="s">
+      <c r="K3" s="2" t="s">
         <v>97</v>
       </c>
     </row>

</xml_diff>